<commit_message>
Caching system, year structure update, formula verification
- Fixed critical backend reactivity that caused data inconsistency by adding a dictionary-based cache to store calculated values throughout current file. New system ensures latest data is used across formulas without multiple file iterations needed  to reach final results.
- Removed "baseline" year zero - now direct year range for cleaner structure and new version actualization
- Verified all formula definitions across sections (except design capital/financial statements WIP)

Cache system prevents reaccesing static file, significantly improving performance.
</commit_message>
<xml_diff>
--- a/backend/LPG testing/carbon-credits-general.xlsx
+++ b/backend/LPG testing/carbon-credits-general.xlsx
@@ -502,7 +502,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O16"/>
+  <dimension ref="A1:O20"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5"/>
   <cols>
     <col width="59.54296875" customWidth="1" min="1" max="1"/>
@@ -662,7 +662,7 @@
     <row r="4" ht="15.5" customHeight="1">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>CO2 emited - Aligned scenario</t>
+          <t>CO2 emited - probar BASELINEEE scenario</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
@@ -711,7 +711,7 @@
     <row r="5" ht="15.5" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>CO2 emited - CleanStep scenario</t>
+          <t>CO2 emited - Aligned scenario</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
@@ -720,47 +720,47 @@
         </is>
       </c>
       <c r="C5" s="13" t="n">
-        <v>21.61054123063169</v>
+        <v>0</v>
       </c>
       <c r="D5" s="13" t="n">
-        <v>19.40524688334832</v>
+        <v>0</v>
       </c>
       <c r="E5" s="13" t="n">
-        <v>17.42849567827935</v>
+        <v>0</v>
       </c>
       <c r="F5" s="13" t="n">
-        <v>15.45174447321038</v>
+        <v>0</v>
       </c>
       <c r="G5" s="13" t="n">
-        <v>13.47499326814141</v>
+        <v>0</v>
       </c>
       <c r="H5" s="13" t="n">
-        <v>11.49824206307243</v>
+        <v>0</v>
       </c>
       <c r="I5" s="13" t="n">
-        <v>9.521490858003462</v>
+        <v>0</v>
       </c>
       <c r="J5" s="13" t="n">
-        <v>9.104909776724984</v>
+        <v>0</v>
       </c>
       <c r="K5" s="13" t="n">
-        <v>9.190097029539562</v>
+        <v>0</v>
       </c>
       <c r="L5" s="13" t="n">
-        <v>9.275284282354139</v>
+        <v>0</v>
       </c>
       <c r="M5" s="13" t="n">
-        <v>9.360471535168717</v>
+        <v>0</v>
       </c>
       <c r="N5" s="13" t="n">
-        <v>9.445658787983295</v>
+        <v>0</v>
       </c>
       <c r="O5" s="8" t="n"/>
     </row>
     <row r="6" ht="15.5" customHeight="1">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>△▲{model} vs. BAU</t>
+          <t>CO2 emited - CleanStep scenario</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
@@ -769,47 +769,47 @@
         </is>
       </c>
       <c r="C6" s="13" t="n">
-        <v>0</v>
+        <v>21.61054123063169</v>
       </c>
       <c r="D6" s="13" t="n">
-        <v>0</v>
+        <v>19.40524688334832</v>
       </c>
       <c r="E6" s="13" t="n">
-        <v>0</v>
+        <v>17.42849567827935</v>
       </c>
       <c r="F6" s="13" t="n">
-        <v>0</v>
+        <v>15.45174447321038</v>
       </c>
       <c r="G6" s="13" t="n">
-        <v>0</v>
+        <v>13.47499326814141</v>
       </c>
       <c r="H6" s="13" t="n">
-        <v>0</v>
+        <v>11.49824206307243</v>
       </c>
       <c r="I6" s="13" t="n">
-        <v>0</v>
+        <v>9.521490858003462</v>
       </c>
       <c r="J6" s="13" t="n">
-        <v>0</v>
+        <v>9.104909776724984</v>
       </c>
       <c r="K6" s="13" t="n">
-        <v>0</v>
+        <v>9.190097029539562</v>
       </c>
       <c r="L6" s="13" t="n">
-        <v>0</v>
+        <v>9.275284282354139</v>
       </c>
       <c r="M6" s="13" t="n">
-        <v>0</v>
+        <v>9.360471535168717</v>
       </c>
       <c r="N6" s="13" t="n">
-        <v>0</v>
+        <v>9.445658787983295</v>
       </c>
       <c r="O6" s="8" t="n"/>
     </row>
     <row r="7" ht="15.5" customHeight="1">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>△▲Aligned vs. BAU</t>
+          <t>△▲{model} vs. BAU</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
@@ -818,47 +818,47 @@
         </is>
       </c>
       <c r="C7" s="13" t="n">
-        <v>21.61017358638736</v>
+        <v>0</v>
       </c>
       <c r="D7" s="13" t="n">
-        <v>20.60189269210638</v>
+        <v>0</v>
       </c>
       <c r="E7" s="13" t="n">
-        <v>19.83817666585722</v>
+        <v>0</v>
       </c>
       <c r="F7" s="13" t="n">
-        <v>19.07446063960807</v>
+        <v>0</v>
       </c>
       <c r="G7" s="13" t="n">
-        <v>18.31074461335891</v>
+        <v>0</v>
       </c>
       <c r="H7" s="13" t="n">
-        <v>17.54702858710975</v>
+        <v>0</v>
       </c>
       <c r="I7" s="13" t="n">
-        <v>16.7833125608606</v>
+        <v>0</v>
       </c>
       <c r="J7" s="13" t="n">
-        <v>16.43569213193877</v>
+        <v>0</v>
       </c>
       <c r="K7" s="13" t="n">
-        <v>16.3666828952225</v>
+        <v>0</v>
       </c>
       <c r="L7" s="13" t="n">
-        <v>16.29767365850622</v>
+        <v>0</v>
       </c>
       <c r="M7" s="13" t="n">
-        <v>16.22866442178994</v>
+        <v>0</v>
       </c>
       <c r="N7" s="13" t="n">
-        <v>16.15965518507367</v>
+        <v>0</v>
       </c>
       <c r="O7" s="8" t="n"/>
     </row>
     <row r="8" ht="15.5" customHeight="1">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>△▲CleanStep vs. BAU</t>
+          <t>△▲probar BASELINEEE vs. BAU</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
@@ -867,47 +867,47 @@
         </is>
       </c>
       <c r="C8" s="13" t="n">
-        <v>-0.0003676442443278916</v>
+        <v>0</v>
       </c>
       <c r="D8" s="13" t="n">
-        <v>1.19664580875806</v>
+        <v>0</v>
       </c>
       <c r="E8" s="13" t="n">
-        <v>2.409680987577868</v>
+        <v>0</v>
       </c>
       <c r="F8" s="13" t="n">
-        <v>3.622716166397689</v>
+        <v>0</v>
       </c>
       <c r="G8" s="13" t="n">
-        <v>4.835751345217499</v>
+        <v>0</v>
       </c>
       <c r="H8" s="13" t="n">
-        <v>6.04878652403732</v>
+        <v>0</v>
       </c>
       <c r="I8" s="13" t="n">
-        <v>7.261821702857139</v>
+        <v>0</v>
       </c>
       <c r="J8" s="13" t="n">
-        <v>7.330782355213785</v>
+        <v>0</v>
       </c>
       <c r="K8" s="13" t="n">
-        <v>7.176585865682938</v>
+        <v>0</v>
       </c>
       <c r="L8" s="13" t="n">
-        <v>7.022389376152081</v>
+        <v>0</v>
       </c>
       <c r="M8" s="13" t="n">
-        <v>6.868192886621223</v>
+        <v>0</v>
       </c>
       <c r="N8" s="13" t="n">
-        <v>6.713996397090376</v>
+        <v>0</v>
       </c>
       <c r="O8" s="8" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>CO2 equivalent avoided in the {model}</t>
+          <t>△▲Aligned vs. BAU</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
@@ -916,47 +916,47 @@
         </is>
       </c>
       <c r="C9" s="13" t="n">
-        <v>0</v>
+        <v>21.61017358638736</v>
       </c>
       <c r="D9" s="13" t="n">
-        <v>0</v>
+        <v>20.60189269210638</v>
       </c>
       <c r="E9" s="13" t="n">
-        <v>0</v>
+        <v>19.83817666585722</v>
       </c>
       <c r="F9" s="13" t="n">
-        <v>0</v>
+        <v>19.07446063960807</v>
       </c>
       <c r="G9" s="13" t="n">
-        <v>0</v>
+        <v>18.31074461335891</v>
       </c>
       <c r="H9" s="13" t="n">
-        <v>0</v>
+        <v>17.54702858710975</v>
       </c>
       <c r="I9" s="13" t="n">
-        <v>0</v>
+        <v>16.7833125608606</v>
       </c>
       <c r="J9" s="13" t="n">
-        <v>0</v>
+        <v>16.43569213193877</v>
       </c>
       <c r="K9" s="13" t="n">
-        <v>0</v>
+        <v>16.3666828952225</v>
       </c>
       <c r="L9" s="13" t="n">
-        <v>0</v>
+        <v>16.29767365850622</v>
       </c>
       <c r="M9" s="13" t="n">
-        <v>0</v>
+        <v>16.22866442178994</v>
       </c>
       <c r="N9" s="13" t="n">
-        <v>0</v>
+        <v>16.15965518507367</v>
       </c>
       <c r="O9" s="8" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>CO2 equivalent avoided in the Aligned</t>
+          <t>△▲CleanStep vs. BAU</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
@@ -965,47 +965,47 @@
         </is>
       </c>
       <c r="C10" s="13" t="n">
-        <v>17.28813886910989</v>
+        <v>-0.0003676442443278916</v>
       </c>
       <c r="D10" s="13" t="n">
-        <v>16.4815141536851</v>
+        <v>1.19664580875806</v>
       </c>
       <c r="E10" s="13" t="n">
-        <v>15.87054133268578</v>
+        <v>2.409680987577868</v>
       </c>
       <c r="F10" s="13" t="n">
-        <v>15.25956851168646</v>
+        <v>3.622716166397689</v>
       </c>
       <c r="G10" s="13" t="n">
-        <v>14.64859569068713</v>
+        <v>4.835751345217499</v>
       </c>
       <c r="H10" s="13" t="n">
-        <v>14.0376228696878</v>
+        <v>6.04878652403732</v>
       </c>
       <c r="I10" s="13" t="n">
-        <v>13.42665004868848</v>
+        <v>7.261821702857139</v>
       </c>
       <c r="J10" s="13" t="n">
-        <v>13.14855370555101</v>
+        <v>7.330782355213785</v>
       </c>
       <c r="K10" s="13" t="n">
-        <v>13.093346316178</v>
+        <v>7.176585865682938</v>
       </c>
       <c r="L10" s="13" t="n">
-        <v>13.03813892680498</v>
+        <v>7.022389376152081</v>
       </c>
       <c r="M10" s="13" t="n">
-        <v>12.98293153743195</v>
+        <v>6.868192886621223</v>
       </c>
       <c r="N10" s="13" t="n">
-        <v>12.92772414805894</v>
+        <v>6.713996397090376</v>
       </c>
       <c r="O10" s="8" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>CO2 equivalent avoided in the CleanStep</t>
+          <t>CO2 equivalent avoided in the {model}</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
@@ -1017,49 +1017,49 @@
         <v>0</v>
       </c>
       <c r="D11" s="13" t="n">
-        <v>0.957316647006448</v>
+        <v>0</v>
       </c>
       <c r="E11" s="13" t="n">
-        <v>1.927744790062295</v>
+        <v>0</v>
       </c>
       <c r="F11" s="13" t="n">
-        <v>2.898172933118151</v>
+        <v>0</v>
       </c>
       <c r="G11" s="13" t="n">
-        <v>3.868601076174</v>
+        <v>0</v>
       </c>
       <c r="H11" s="13" t="n">
-        <v>4.839029219229856</v>
+        <v>0</v>
       </c>
       <c r="I11" s="13" t="n">
-        <v>5.809457362285712</v>
+        <v>0</v>
       </c>
       <c r="J11" s="13" t="n">
-        <v>5.864625884171028</v>
+        <v>0</v>
       </c>
       <c r="K11" s="13" t="n">
-        <v>5.741268692546351</v>
+        <v>0</v>
       </c>
       <c r="L11" s="13" t="n">
-        <v>5.617911500921664</v>
+        <v>0</v>
       </c>
       <c r="M11" s="13" t="n">
-        <v>5.494554309296978</v>
+        <v>0</v>
       </c>
       <c r="N11" s="13" t="n">
-        <v>5.371197117672301</v>
+        <v>0</v>
       </c>
       <c r="O11" s="8" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>Potential income from Carbon Credits in the {model} Plan - right</t>
+          <t>CO2 equivalent avoided in the probar BASELINEEE</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>M USD</t>
+          <t>CO2Eq MT/y</t>
         </is>
       </c>
       <c r="C12" s="13" t="n">
@@ -1103,130 +1103,326 @@
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>Potential income from Carbon Credits in the Aligned Plan - right</t>
+          <t>CO2 equivalent avoided in the Aligned</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>M USD</t>
+          <t>CO2Eq MT/y</t>
         </is>
       </c>
       <c r="C13" s="13" t="n">
-        <v>172.8813886910989</v>
+        <v>0</v>
       </c>
       <c r="D13" s="13" t="n">
-        <v>164.815141536851</v>
+        <v>0</v>
       </c>
       <c r="E13" s="13" t="n">
-        <v>158.7054133268578</v>
+        <v>0</v>
       </c>
       <c r="F13" s="13" t="n">
-        <v>152.5956851168646</v>
+        <v>0</v>
       </c>
       <c r="G13" s="13" t="n">
-        <v>146.4859569068713</v>
+        <v>0</v>
       </c>
       <c r="H13" s="13" t="n">
-        <v>140.376228696878</v>
+        <v>0</v>
       </c>
       <c r="I13" s="13" t="n">
-        <v>134.2665004868848</v>
+        <v>0</v>
       </c>
       <c r="J13" s="13" t="n">
-        <v>131.4855370555101</v>
+        <v>0</v>
       </c>
       <c r="K13" s="13" t="n">
-        <v>130.93346316178</v>
+        <v>0</v>
       </c>
       <c r="L13" s="13" t="n">
-        <v>130.3813892680498</v>
+        <v>0</v>
       </c>
       <c r="M13" s="13" t="n">
-        <v>129.8293153743195</v>
+        <v>0</v>
       </c>
       <c r="N13" s="13" t="n">
-        <v>129.2772414805894</v>
+        <v>0</v>
       </c>
       <c r="O13" s="8" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
         <is>
+          <t>CO2 equivalent avoided in the CleanStep</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>CO2Eq MT/y</t>
+        </is>
+      </c>
+      <c r="C14" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="D14" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="E14" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="F14" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="G14" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="H14" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="I14" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="J14" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="K14" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="L14" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="M14" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="N14" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="O14" s="8" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>Potential income from Carbon Credits in the {model} Plan - right</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>M USD</t>
+        </is>
+      </c>
+      <c r="C15" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="D15" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="E15" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="F15" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="G15" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="H15" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="I15" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="J15" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="K15" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="L15" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="M15" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="N15" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="O15" s="8" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Potential income from Carbon Credits in the probar BASELINEEE Plan - right</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>M USD</t>
+        </is>
+      </c>
+      <c r="C16" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="D16" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="E16" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="F16" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="G16" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="H16" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="I16" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="J16" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="K16" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="L16" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="M16" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="N16" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="O16" s="8" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>Potential income from Carbon Credits in the Aligned Plan - right</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>M USD</t>
+        </is>
+      </c>
+      <c r="C17" s="13" t="n">
+        <v>172.8813886910989</v>
+      </c>
+      <c r="D17" s="13" t="n">
+        <v>164.815141536851</v>
+      </c>
+      <c r="E17" s="13" t="n">
+        <v>158.7054133268578</v>
+      </c>
+      <c r="F17" s="13" t="n">
+        <v>152.5956851168646</v>
+      </c>
+      <c r="G17" s="13" t="n">
+        <v>146.4859569068713</v>
+      </c>
+      <c r="H17" s="13" t="n">
+        <v>140.376228696878</v>
+      </c>
+      <c r="I17" s="13" t="n">
+        <v>134.2665004868848</v>
+      </c>
+      <c r="J17" s="13" t="n">
+        <v>131.4855370555101</v>
+      </c>
+      <c r="K17" s="13" t="n">
+        <v>130.93346316178</v>
+      </c>
+      <c r="L17" s="13" t="n">
+        <v>130.3813892680498</v>
+      </c>
+      <c r="M17" s="13" t="n">
+        <v>129.8293153743195</v>
+      </c>
+      <c r="N17" s="13" t="n">
+        <v>129.2772414805894</v>
+      </c>
+      <c r="O17" s="8" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
           <t>Potential income from Carbon Credits in the CleanStep Plan - right</t>
         </is>
       </c>
-      <c r="B14" s="3" t="inlineStr">
+      <c r="B18" s="3" t="inlineStr">
         <is>
           <t>M USD</t>
         </is>
       </c>
-      <c r="C14" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="D14" s="13" t="n">
+      <c r="C18" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="D18" s="13" t="n">
         <v>9.57316647006448</v>
       </c>
-      <c r="E14" s="13" t="n">
+      <c r="E18" s="13" t="n">
         <v>19.27744790062295</v>
       </c>
-      <c r="F14" s="13" t="n">
+      <c r="F18" s="13" t="n">
         <v>28.98172933118151</v>
       </c>
-      <c r="G14" s="13" t="n">
+      <c r="G18" s="13" t="n">
         <v>38.68601076174</v>
       </c>
-      <c r="H14" s="13" t="n">
+      <c r="H18" s="13" t="n">
         <v>48.39029219229856</v>
       </c>
-      <c r="I14" s="13" t="n">
+      <c r="I18" s="13" t="n">
         <v>58.09457362285712</v>
       </c>
-      <c r="J14" s="13" t="n">
+      <c r="J18" s="13" t="n">
         <v>58.64625884171028</v>
       </c>
-      <c r="K14" s="13" t="n">
+      <c r="K18" s="13" t="n">
         <v>57.4126869254635</v>
       </c>
-      <c r="L14" s="13" t="n">
+      <c r="L18" s="13" t="n">
         <v>56.17911500921664</v>
       </c>
-      <c r="M14" s="13" t="n">
+      <c r="M18" s="13" t="n">
         <v>54.94554309296979</v>
       </c>
-      <c r="N14" s="13" t="n">
+      <c r="N18" s="13" t="n">
         <v>53.71197117672301</v>
       </c>
-      <c r="O14" s="8" t="n"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="9" t="n"/>
-      <c r="B15" s="1" t="n"/>
-      <c r="C15" s="1" t="n"/>
-      <c r="D15" s="10" t="n"/>
-      <c r="E15" s="10" t="n"/>
-      <c r="F15" s="10" t="n"/>
-      <c r="G15" s="10" t="n"/>
-      <c r="H15" s="10" t="n"/>
-      <c r="I15" s="10" t="n"/>
-      <c r="J15" s="10" t="n"/>
-      <c r="K15" s="10" t="n"/>
-      <c r="L15" s="10" t="n"/>
-      <c r="M15" s="10" t="n"/>
-      <c r="N15" s="10" t="n"/>
-      <c r="O15" s="8" t="n"/>
-    </row>
-    <row r="16">
-      <c r="A16" s="2" t="n"/>
-      <c r="B16" s="1" t="n"/>
-      <c r="C16" s="1" t="n"/>
-      <c r="D16" s="2" t="n"/>
-      <c r="E16" s="2" t="n"/>
-      <c r="F16" s="2" t="n"/>
-      <c r="G16" s="2" t="n"/>
-      <c r="H16" s="2" t="n"/>
-      <c r="I16" s="2" t="n"/>
-      <c r="J16" s="2" t="n"/>
-      <c r="K16" s="2" t="n"/>
+      <c r="O18" s="8" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="9" t="n"/>
+      <c r="B19" s="1" t="n"/>
+      <c r="C19" s="1" t="n"/>
+      <c r="D19" s="10" t="n"/>
+      <c r="E19" s="10" t="n"/>
+      <c r="F19" s="10" t="n"/>
+      <c r="G19" s="10" t="n"/>
+      <c r="H19" s="10" t="n"/>
+      <c r="I19" s="10" t="n"/>
+      <c r="J19" s="10" t="n"/>
+      <c r="K19" s="10" t="n"/>
+      <c r="L19" s="10" t="n"/>
+      <c r="M19" s="10" t="n"/>
+      <c r="N19" s="10" t="n"/>
+      <c r="O19" s="8" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="n"/>
+      <c r="B20" s="1" t="n"/>
+      <c r="C20" s="1" t="n"/>
+      <c r="D20" s="2" t="n"/>
+      <c r="E20" s="2" t="n"/>
+      <c r="F20" s="2" t="n"/>
+      <c r="G20" s="2" t="n"/>
+      <c r="H20" s="2" t="n"/>
+      <c r="I20" s="2" t="n"/>
+      <c r="J20" s="2" t="n"/>
+      <c r="K20" s="2" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>